<commit_message>
Added first card from deck
</commit_message>
<xml_diff>
--- a/Assets/Docs/Protocol.xlsx
+++ b/Assets/Docs/Protocol.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="76" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DAE770B-0F94-466C-B35D-FEE597E5F3EA}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\storage\unity games\Year 2\Semester 2\Networking\NetworkingProject\Assets\Docs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A586CAB3-771A-4856-8D60-A44DFA69C47B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="3405" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="28">
   <si>
     <t>Client -&gt; Server</t>
   </si>
@@ -81,9 +86,6 @@
     <t>DrawCard</t>
   </si>
   <si>
-    <t>PlayerDrewCard</t>
-  </si>
-  <si>
     <t>player</t>
   </si>
   <si>
@@ -112,13 +114,19 @@
   </si>
   <si>
     <t>SetDrawnCards</t>
+  </si>
+  <si>
+    <t>SetFirstCard</t>
+  </si>
+  <si>
+    <t>PlayerDrewCards</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -199,9 +207,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -239,7 +247,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -345,7 +353,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -487,7 +495,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -495,14 +503,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:M16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.28515625" customWidth="1"/>
     <col min="7" max="7" width="18.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -514,7 +522,7 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -534,7 +542,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" s="3" t="s">
         <v>5</v>
@@ -553,7 +561,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -576,90 +584,104 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>15</v>
       </c>
       <c r="G5" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="H5" t="s">
         <v>9</v>
       </c>
       <c r="I5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H6" t="s">
         <v>9</v>
       </c>
       <c r="I6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="G7" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="G7" t="s">
-        <v>20</v>
       </c>
       <c r="H7" t="s">
         <v>9</v>
       </c>
       <c r="I7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="G8" t="s">
+        <v>26</v>
+      </c>
+      <c r="H8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I8" t="s">
+        <v>13</v>
+      </c>
+      <c r="J8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="G13" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="G9" t="s">
+      <c r="H13" t="s">
+        <v>9</v>
+      </c>
+      <c r="I13" t="s">
         <v>22</v>
       </c>
-      <c r="H9" t="s">
+      <c r="J13" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="H14" t="s">
+        <v>12</v>
+      </c>
+      <c r="I14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="G15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H15" t="s">
         <v>9</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I15" t="s">
+        <v>22</v>
+      </c>
+      <c r="J15" t="s">
         <v>23</v>
       </c>
-      <c r="J9" t="s">
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="H16" t="s">
+        <v>12</v>
+      </c>
+      <c r="I16" t="s">
         <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="H10" t="s">
-        <v>12</v>
-      </c>
-      <c r="I10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13">
-      <c r="G11" t="s">
-        <v>26</v>
-      </c>
-      <c r="H11" t="s">
-        <v>9</v>
-      </c>
-      <c r="I11" t="s">
-        <v>23</v>
-      </c>
-      <c r="J11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13">
-      <c r="H12" t="s">
-        <v>12</v>
-      </c>
-      <c r="I12" t="s">
-        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Player cannow draw cards properly
still need to advance game after the cards being drawn
</commit_message>
<xml_diff>
--- a/Assets/Docs/Protocol.xlsx
+++ b/Assets/Docs/Protocol.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\storage\unity games\Year 2\Semester 2\Networking\NetworkingProject\Assets\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A8A5F0D-FCA4-4D8E-9E0E-5B68E8743950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74D17558-3C54-4A58-82BA-34EFD97C6EF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="3405" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="29">
   <si>
     <t>Client -&gt; Server</t>
   </si>
@@ -119,7 +119,10 @@
     <t>SetFirstCard</t>
   </si>
   <si>
-    <t>PlayerDrewCards</t>
+    <t>PlayerDrawCards</t>
+  </si>
+  <si>
+    <t>note that player int is only used in the event from the model</t>
   </si>
 </sst>
 </file>
@@ -661,6 +664,9 @@
       <c r="J11" t="s">
         <v>23</v>
       </c>
+      <c r="K11" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="H12" t="s">

</xml_diff>